<commit_message>
changes in clame excel
</commit_message>
<xml_diff>
--- a/claim.xlsx
+++ b/claim.xlsx
@@ -1,69 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\newproj\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652239BB-7480-4B03-B9FE-D8AB130D98E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>Employee_Code</t>
-  </si>
-  <si>
-    <t>Invoice_No</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Total_Amount</t>
-  </si>
-  <si>
-    <t>Claim_Type</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -71,44 +42,85 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -396,25 +408,214 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Employee_Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Invoice_No</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Total_Amount</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Claim_Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>5M/2019-20/168</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2019-09-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>567</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>626</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>615</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>INV-002</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INV-003</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>30</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>INV-004</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes in clame excel 1
</commit_message>
<xml_diff>
--- a/claim.xlsx
+++ b/claim.xlsx
@@ -1,81 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\newproj\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A49DAE-BF28-4648-8C87-2D66E68D24B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>Employee_Code</t>
-  </si>
-  <si>
-    <t>Invoice_No</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Total_Amount</t>
-  </si>
-  <si>
-    <t>Claim_Type</t>
-  </si>
-  <si>
-    <t>Claim_ID</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -83,47 +42,85 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -411,35 +408,263 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="5" max="5" width="17.08984375" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Employee_Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Invoice_No</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Total_Amount</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Claim_Type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Claim_ID</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>5M/2019-20/168</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2019-09-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>567</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1234321</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>626</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1234321</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>615</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1234321</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>INV-002</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INV-003</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>30</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>INV-004</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
changes in clame excel 2
</commit_message>
<xml_diff>
--- a/claim.xlsx
+++ b/claim.xlsx
@@ -1,81 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\newproj\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A49DAE-BF28-4648-8C87-2D66E68D24B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>Employee_Code</t>
-  </si>
-  <si>
-    <t>Invoice_No</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Total_Amount</t>
-  </si>
-  <si>
-    <t>Claim_Type</t>
-  </si>
-  <si>
-    <t>Claim_ID</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -83,47 +42,85 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -411,34 +408,294 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="5" max="5" width="17.08984375" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Employee_Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Invoice_No</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Total_Amount</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Claim_Type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Claim_ID</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>5M/2019-20/168</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2019-09-25</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>567</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>626</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>615</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>INV-002</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INV-003</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>30</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>INV-004</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sent temp file also
</commit_message>
<xml_diff>
--- a/claim.xlsx
+++ b/claim.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2401,6 +2401,2211 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>5M/2019-20/168</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2019-09-25</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>567</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2f943a4f-8caf-4203-a568-baa86db71969</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>626</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>5ab2aecc-bb06-4f18-87e2-975f54492d0c</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>615</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>aa214bf8-b8ab-4e23-8b27-985681d39f42</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>10</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>56daefd5-2704-40ae-bbe0-4020ded8b88d</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>INV-002</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>20</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>1e779ef5-a01f-4606-bd49-6222dd74c23e</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>INV-003</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>30</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>a2e7c350-7ab6-4d73-b0cf-118f35b8ead6</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>INV-004</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>40</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>f1f00255-4051-43bb-9197-31895f546a05</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>5M/2019-20/168</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2019-09-25</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>567</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>75f79aa8-2fe0-4b3b-ad07-34a22979924d</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>626</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>518319cc-c746-4ae9-b363-d855fb79ff39</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>615</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>d459a79b-fce7-48c3-bb38-882bf8a50d45</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>10</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>0dcf9ffc-9351-4a88-bf21-448e6fa267a9</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>INV-002</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>20</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>64bae692-a8f6-405e-93a3-fa66a3ea7f1a</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>INV-003</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>30</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>113865a3-4619-46f7-80f2-eeae49cfbef8</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>INV-004</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>40</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>815ad0b0-1a68-402f-9d55-ce2d95bd4065</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>5M/2019-20/168</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2019-09-25</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>567</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2dd16fe3-e0aa-4813-b00c-49b6ab9e711e</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>626</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>36a00c1b-18ab-4f79-b90c-fc8bb2075bc9</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>615</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>ae79eec4-1543-42a3-a9e8-31719ac703a3</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>10</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>e348217e-a8f8-4990-8deb-8d68ccb70a54</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>INV-002</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>20</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>9a6adb29-5e49-4b85-aafd-721f9802f2a9</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>INV-003</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>30</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>5ce473c7-0f83-40d6-9479-bd4ba396d5ff</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>INV-004</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>40</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>28a108cb-9a56-422a-b011-37ec02d88dc1</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>5M/2019-20/168</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2019-09-25</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>567</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>1bf43312-769a-4c1f-8fab-aa6bd8bdfde1</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>626</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>a2a063d0-3b20-4821-bf7e-286dfe5679f9</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>615</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>7e91f163-e470-400b-b6bc-dda59427ca19</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>10</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>0e1a8cdc-eaa7-469a-98ea-34d0c922fbfe</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>INV-002</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>20</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>4876a54c-07d8-4783-a49f-3e24ac56940b</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>INV-003</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>30</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>dd178dfc-28cc-4c6c-934e-15e41a0ddeb6</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>INV-004</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>40</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>8ef8e720-60f4-4c6e-9107-43246581f3d9</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>5M/2019-20/168</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2019-09-25</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>567</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>010df1b1-d243-4154-bc21-dbac66c6fc03</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>626</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>a9497c0e-de11-4470-a142-72aac0e20c87</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>615</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>cac091ae-d86c-4a25-a06b-7b1f52f1440b</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>10</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>7b431da8-e4d3-4882-b6be-74b660e7a482</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>INV-002</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>20</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>7765299d-aee4-407e-adc8-1258c866115f</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>INV-003</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>30</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>43b63f2d-f084-4018-b03d-93624fbc335a</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>INV-004</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>40</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>2354d85b-8591-4be0-aa1a-846a41f66336</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>5M/2019-20/168</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2019-09-25</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>567</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>138a3cec-d579-430a-9596-b8c8ce9c9380</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>626</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>4d4dc4fd-6cc0-4682-9c6f-3f09426555a7</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>615</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>ae2b8caa-0a8b-4f44-9c08-0327f317a21c</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>10</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>d6e92c11-d552-48b0-bcca-cc77d722d682</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>INV-002</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>20</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>300307eb-84b1-42c5-bdd9-033d02dd6679</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>INV-003</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>30</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>bc287a02-8915-4718-897c-cab5d65b58ba</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>INV-004</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>40</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>64c894ba-39ac-4055-b51e-e999d3379e65</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>5M/2019-20/168</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2019-09-25</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>567</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>b3425f2c-ba73-443e-944a-a78afe8842ab</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2024-04-03</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>626</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>22dceb18-fe97-4b65-ba0d-9d04402ce647</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Invoice Not Found</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>2024-04-04</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>615</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Individual_Expense</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>12403d80-13d7-4238-9aad-4c13d3d1f6c5</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>10</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>11dfa7c7-6d77-40d9-b25a-fcc5599253c7</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>INV-002</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>20</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>a90b663d-6021-45be-974a-9f3c4c864eef</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>INV-003</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>30</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>00df8bd5-4be2-4243-89c4-e998682553af</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>E-0001</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>INV-004</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>40</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Daily_Expense</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>CL_230022</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>fb6ad48d-e2a6-42f7-960a-4043c78619f0</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>